<commit_message>
update client portal data
</commit_message>
<xml_diff>
--- a/clientportal/Contracts and Amendments - 4871_OC-CR.xlsx
+++ b/clientportal/Contracts and Amendments - 4871_OC-CR.xlsx
@@ -664,6 +664,18 @@
   </si>
   <si>
     <t>Plazo definido </t>
+  </si>
+  <si>
+    <t>CR-L1137-P00408</t>
+  </si>
+  <si>
+    <t>4871OCCR-CR-L1137-P00408-C01</t>
+  </si>
+  <si>
+    <t>Contratación de servicios profesionales como Autoridad de Probidad Independiente (API) 3 para la conclusión de 4 Centros Cívicos por la Paz de Pérez Zeledón, San José, Goicoechea y Liberia.</t>
+  </si>
+  <si>
+    <t>Randall Muñoz Matamoros</t>
   </si>
   <si>
     <t>Componente 2: Prevención social de la violencia</t>
@@ -1095,7 +1107,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI24"/>
+  <dimension ref="A1:AI25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="18.6640625" style="1" customWidth="1"/>
@@ -3180,6 +3192,89 @@
       <c r="AH24" s="2"/>
       <c r="AI24" s="4"/>
     </row>
+    <row r="25" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A25" t="s" s="1">
+        <v>213</v>
+      </c>
+      <c r="B25" t="s" s="1">
+        <v>214</v>
+      </c>
+      <c r="C25" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="D25" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="E25" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="F25" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="G25" t="s" s="1">
+        <v>121</v>
+      </c>
+      <c r="H25" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="I25" s="2"/>
+      <c r="J25" t="s" s="1">
+        <v>123</v>
+      </c>
+      <c r="K25" t="n" s="6">
+        <v>46293</v>
+      </c>
+      <c r="L25" t="n" s="6">
+        <v>46294</v>
+      </c>
+      <c r="M25" t="n" s="6">
+        <v>46446</v>
+      </c>
+      <c r="N25" t="s" s="1">
+        <v>124</v>
+      </c>
+      <c r="O25" t="n" s="3">
+        <v>30000</v>
+      </c>
+      <c r="P25" t="n" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n" s="3">
+        <v>0</v>
+      </c>
+      <c r="R25" t="n" s="3">
+        <v>30000</v>
+      </c>
+      <c r="S25" s="2"/>
+      <c r="T25" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="U25" s="2"/>
+      <c r="V25" t="n" s="2">
+        <v>9968</v>
+      </c>
+      <c r="W25" t="s" s="2">
+        <v>126</v>
+      </c>
+      <c r="X25" t="s" s="2">
+        <v>127</v>
+      </c>
+      <c r="Y25" s="2"/>
+      <c r="Z25" t="n" s="1">
+        <v>10101</v>
+      </c>
+      <c r="AA25" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="AB25" s="2"/>
+      <c r="AC25" s="4"/>
+      <c r="AD25" s="2"/>
+      <c r="AE25" s="4"/>
+      <c r="AF25" s="2"/>
+      <c r="AG25" s="4"/>
+      <c r="AH25" s="2"/>
+      <c r="AI25" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3187,7 +3282,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.6640625" style="1" customWidth="1"/>
@@ -3251,10 +3346,10 @@
         <v>118</v>
       </c>
       <c r="E2" t="s" s="2">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="F2" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="G2" t="s" s="1">
         <v>124</v>
@@ -3286,10 +3381,10 @@
         <v>130</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="F3" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="G3" t="s" s="1">
         <v>124</v>
@@ -3321,10 +3416,10 @@
         <v>134</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="F4" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="G4" t="s" s="1">
         <v>124</v>
@@ -3356,10 +3451,10 @@
         <v>138</v>
       </c>
       <c r="E5" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F5" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G5" t="s" s="1">
         <v>124</v>
@@ -3391,10 +3486,10 @@
         <v>143</v>
       </c>
       <c r="E6" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F6" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G6" t="s" s="1">
         <v>124</v>
@@ -3426,10 +3521,10 @@
         <v>147</v>
       </c>
       <c r="E7" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F7" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G7" t="s" s="1">
         <v>124</v>
@@ -3461,10 +3556,10 @@
         <v>150</v>
       </c>
       <c r="E8" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F8" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G8" t="s" s="1">
         <v>124</v>
@@ -3496,10 +3591,10 @@
         <v>153</v>
       </c>
       <c r="E9" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F9" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G9" t="s" s="1">
         <v>124</v>
@@ -3531,10 +3626,10 @@
         <v>156</v>
       </c>
       <c r="E10" t="s" s="2">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="F10" t="s" s="2">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="G10" t="s" s="1">
         <v>124</v>
@@ -3566,10 +3661,10 @@
         <v>160</v>
       </c>
       <c r="E11" t="s" s="2">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="F11" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="G11" t="s" s="1">
         <v>124</v>
@@ -3601,10 +3696,10 @@
         <v>163</v>
       </c>
       <c r="E12" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F12" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G12" t="s" s="1">
         <v>124</v>
@@ -3636,10 +3731,10 @@
         <v>166</v>
       </c>
       <c r="E13" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F13" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G13" t="s" s="1">
         <v>124</v>
@@ -3671,10 +3766,10 @@
         <v>169</v>
       </c>
       <c r="E14" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F14" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G14" t="s" s="1">
         <v>124</v>
@@ -3706,10 +3801,10 @@
         <v>177</v>
       </c>
       <c r="E15" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F15" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G15" t="s" s="1">
         <v>124</v>
@@ -3741,10 +3836,10 @@
         <v>181</v>
       </c>
       <c r="E16" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F16" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G16" t="s" s="1">
         <v>183</v>
@@ -3776,10 +3871,10 @@
         <v>186</v>
       </c>
       <c r="E17" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F17" t="s" s="2">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="G17" t="s" s="1">
         <v>124</v>
@@ -3811,10 +3906,10 @@
         <v>190</v>
       </c>
       <c r="E18" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F18" t="s" s="2">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="G18" t="s" s="1">
         <v>124</v>
@@ -3846,10 +3941,10 @@
         <v>195</v>
       </c>
       <c r="E19" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F19" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G19" t="s" s="1">
         <v>124</v>
@@ -3881,10 +3976,10 @@
         <v>198</v>
       </c>
       <c r="E20" t="s" s="2">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="F20" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="G20" t="s" s="1">
         <v>124</v>
@@ -3916,10 +4011,10 @@
         <v>203</v>
       </c>
       <c r="E21" t="s" s="2">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="F21" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="G21" t="s" s="1">
         <v>124</v>
@@ -3951,10 +4046,10 @@
         <v>205</v>
       </c>
       <c r="E22" t="s" s="2">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="F22" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="G22" t="s" s="1">
         <v>124</v>
@@ -3986,10 +4081,10 @@
         <v>207</v>
       </c>
       <c r="E23" t="s" s="2">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="F23" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="G23" t="s" s="1">
         <v>124</v>
@@ -4021,10 +4116,10 @@
         <v>210</v>
       </c>
       <c r="E24" t="s" s="2">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="F24" t="s" s="2">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="G24" t="s" s="1">
         <v>124</v>
@@ -4040,6 +4135,41 @@
       </c>
       <c r="K24" t="n" s="3">
         <v>17550</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" t="n" s="1">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s" s="1">
+        <v>213</v>
+      </c>
+      <c r="C25" t="s" s="1">
+        <v>214</v>
+      </c>
+      <c r="D25" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="E25" t="s" s="2">
+        <v>223</v>
+      </c>
+      <c r="F25" t="s" s="2">
+        <v>224</v>
+      </c>
+      <c r="G25" t="s" s="1">
+        <v>124</v>
+      </c>
+      <c r="H25" t="n" s="3">
+        <v>30000</v>
+      </c>
+      <c r="I25" t="n" s="3">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n" s="3">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n" s="3">
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>